<commit_message>
Atualizado casos de testes
</commit_message>
<xml_diff>
--- a/referencias/Casos_de_Teste_Controle_de_Bar_2026.xlsx
+++ b/referencias/Casos_de_Teste_Controle_de_Bar_2026.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Teste" sheetId="1" r:id="R0d45673e189b43ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Teste" sheetId="1" r:id="R28526000c3a14705"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -390,7 +390,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CasosDeTeste" displayName="CasosDeTeste" ref="A1:I103" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CasosDeTeste" displayName="CasosDeTeste" ref="A1:I97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Módulo"/>
@@ -706,7 +706,7 @@
         <x:v>RN-03, RN-04</x:v>
       </x:c>
       <x:c r="I2" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -735,7 +735,7 @@
         <x:v>RN-03</x:v>
       </x:c>
       <x:c r="I3" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -764,7 +764,7 @@
         <x:v>RN-04</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" hidden="0" customHeight="1">
@@ -793,7 +793,7 @@
         <x:v>RN-03, RN-04</x:v>
       </x:c>
       <x:c r="I5" s="15" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -822,7 +822,7 @@
         <x:v>RN-01, RN-03</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -851,7 +851,7 @@
         <x:v>RN-03</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -880,7 +880,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I8" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
@@ -909,7 +909,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" hidden="0" customHeight="1">
@@ -938,7 +938,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -967,7 +967,7 @@
         <x:v>RN-01, RN-02</x:v>
       </x:c>
       <x:c r="I11" s="11" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -996,7 +996,7 @@
         <x:v>RN-05</x:v>
       </x:c>
       <x:c r="I12" s="18" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1025,7 +1025,7 @@
         <x:v>RN-05</x:v>
       </x:c>
       <x:c r="I13" s="18" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
@@ -1054,7 +1054,7 @@
         <x:v>RN-05</x:v>
       </x:c>
       <x:c r="I14" s="22" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -1083,7 +1083,7 @@
         <x:v>RN-01, RN-05</x:v>
       </x:c>
       <x:c r="I15" s="18" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -1112,7 +1112,7 @@
         <x:v>RN-05</x:v>
       </x:c>
       <x:c r="I16" s="18" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1141,7 +1141,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I17" s="18" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" hidden="0" customHeight="1">
@@ -1170,7 +1170,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I18" s="18" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" hidden="0" customHeight="1">
@@ -1199,7 +1199,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I19" s="18" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -1228,7 +1228,7 @@
         <x:v>RN-06, RN-07</x:v>
       </x:c>
       <x:c r="I20" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -1257,7 +1257,7 @@
         <x:v>RN-06</x:v>
       </x:c>
       <x:c r="I21" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -1286,7 +1286,7 @@
         <x:v>RN-07</x:v>
       </x:c>
       <x:c r="I22" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -1315,7 +1315,7 @@
         <x:v>RN-07</x:v>
       </x:c>
       <x:c r="I23" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" hidden="0" customHeight="1">
@@ -1344,7 +1344,7 @@
         <x:v>RN-06, RN-07</x:v>
       </x:c>
       <x:c r="I24" s="29" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -1373,7 +1373,7 @@
         <x:v>RN-01, RN-06</x:v>
       </x:c>
       <x:c r="I25" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" hidden="0" customHeight="1">
@@ -1402,7 +1402,7 @@
         <x:v>RN-06</x:v>
       </x:c>
       <x:c r="I26" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -1431,7 +1431,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I27" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" hidden="0" customHeight="1">
@@ -1460,7 +1460,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I28" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
@@ -1489,7 +1489,7 @@
         <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I29" s="25" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="36" hidden="0" customHeight="1">
@@ -1518,7 +1518,7 @@
         <x:v>RN-12, Funcionalidade: Contas</x:v>
       </x:c>
       <x:c r="I30" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" hidden="0" customHeight="1">
@@ -1547,7 +1547,7 @@
         <x:v>Funcionalidade: Contas</x:v>
       </x:c>
       <x:c r="I31" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
@@ -1576,7 +1576,7 @@
         <x:v>RN-12</x:v>
       </x:c>
       <x:c r="I32" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -1605,7 +1605,7 @@
         <x:v>RN-12</x:v>
       </x:c>
       <x:c r="I33" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
@@ -1634,186 +1634,186 @@
         <x:v>RN-13</x:v>
       </x:c>
       <x:c r="I34" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="32" t="str">
-        <x:v>CT34</x:v>
+        <x:v>CT40</x:v>
       </x:c>
       <x:c r="B35" s="32" t="str">
         <x:v>Conta</x:v>
       </x:c>
       <x:c r="C35" s="32" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D35" s="32" t="str">
-        <x:v>ValorTotal sem pedidos é zero</x:v>
+        <x:v>Abrir conta com dados válidos</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>Conta aberta sem pedidos</x:v>
+        <x:v>Mesa livre, garçom existente, ambos do mesmo UserId</x:v>
       </x:c>
       <x:c r="F35" s="32" t="str">
-        <x:v>Verificar conta.ValorTotal</x:v>
+        <x:v>Chamar Abrir(mesaId, garcomId, "Carlos", userId)</x:v>
       </x:c>
       <x:c r="G35" s="32" t="str">
-        <x:v>ValorTotal == 0m</x:v>
+        <x:v>Result.IsSuccess. Conta persistida. Status=Aberta. DataFechamento=null. Mesa → Ocupada (se era primeira conta)</x:v>
       </x:c>
       <x:c r="H35" s="32" t="str">
-        <x:v>RN-19</x:v>
+        <x:v>RN-01, RN-09, RN-10, RN-12</x:v>
       </x:c>
       <x:c r="I35" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="32" t="str">
-        <x:v>CT35</x:v>
+        <x:v>CT41</x:v>
       </x:c>
       <x:c r="B36" s="32" t="str">
         <x:v>Conta</x:v>
       </x:c>
       <x:c r="C36" s="32" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D36" s="32" t="str">
-        <x:v>ValorTotal soma subtotais</x:v>
+        <x:v>Abrir conta em mesa já ocupada</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>Conta com 2 pedidos: (10x2=20) e (5x3=15)</x:v>
+        <x:v>Mesa ocupada (1 conta aberta existente)</x:v>
       </x:c>
       <x:c r="F36" s="32" t="str">
-        <x:v>Verificar conta.ValorTotal</x:v>
+        <x:v>Chamar Abrir com a mesma mesa</x:v>
       </x:c>
       <x:c r="G36" s="32" t="str">
-        <x:v>ValorTotal == 35m</x:v>
+        <x:v>Result.IsSuccess. Nova conta criada. Mesa permanece Ocupada. Múltiplas contas abertas permitidas</x:v>
       </x:c>
       <x:c r="H36" s="32" t="str">
-        <x:v>RN-19</x:v>
+        <x:v>RN-09, RN-10</x:v>
       </x:c>
       <x:c r="I36" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="32" t="str">
-        <x:v>CT36</x:v>
+        <x:v>CT42</x:v>
       </x:c>
       <x:c r="B37" s="32" t="str">
         <x:v>Conta</x:v>
       </x:c>
       <x:c r="C37" s="32" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D37" s="32" t="str">
-        <x:v>Adicionar pedido em conta aberta</x:v>
+        <x:v>Abrir conta com mesa de outro usuário</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>Conta aberta, pedido válido</x:v>
+        <x:v>Mesa pertence a UserId=B, tentar abrir conta com UserId=A</x:v>
       </x:c>
       <x:c r="F37" s="32" t="str">
-        <x:v>Chamar conta.AdicionarPedido(pedido)</x:v>
+        <x:v>Chamar Abrir com mesaId de B e userId=A</x:v>
       </x:c>
       <x:c r="G37" s="32" t="str">
-        <x:v>Pedido adicionado à lista. Pedidos.Count incrementa</x:v>
+        <x:v>Result.IsFailed. Erro: "Mesa não encontrada para este usuário."</x:v>
       </x:c>
       <x:c r="H37" s="32" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-02, RN-12</x:v>
       </x:c>
       <x:c r="I37" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="32" t="str">
-        <x:v>CT37</x:v>
+        <x:v>CT43</x:v>
       </x:c>
       <x:c r="B38" s="32" t="str">
         <x:v>Conta</x:v>
       </x:c>
       <x:c r="C38" s="32" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D38" s="32" t="str">
-        <x:v>Adicionar pedido em conta fechada lança exceção</x:v>
+        <x:v>Abrir conta com garçom de outro usuário</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>Conta fechada</x:v>
+        <x:v>Garçom pertence a UserId=B, tentar abrir conta com UserId=A</x:v>
       </x:c>
       <x:c r="F38" s="32" t="str">
-        <x:v>Chamar conta.AdicionarPedido(pedido)</x:v>
+        <x:v>Chamar Abrir com garcomId de B e userId=A</x:v>
       </x:c>
       <x:c r="G38" s="32" t="str">
-        <x:v>Lança InvalidOperationException</x:v>
+        <x:v>Result.IsFailed. Erro: "Garçom não encontrado para este usuário."</x:v>
       </x:c>
       <x:c r="H38" s="32" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-02, RN-12</x:v>
       </x:c>
       <x:c r="I38" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="32" t="str">
-        <x:v>CT38</x:v>
+        <x:v>CT44</x:v>
       </x:c>
       <x:c r="B39" s="32" t="str">
         <x:v>Conta</x:v>
       </x:c>
       <x:c r="C39" s="32" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D39" s="32" t="str">
-        <x:v>Remover pedido em conta aberta</x:v>
+        <x:v>Fechar conta preserva total e histórico dos pedidos</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>Conta aberta com 1 pedido</x:v>
+        <x:v>Conta aberta com pedidos e produtos posteriormente editados</x:v>
       </x:c>
       <x:c r="F39" s="32" t="str">
-        <x:v>Chamar conta.RemoverPedido(pedidoId)</x:v>
+        <x:v>Registrar o total. Fechar a conta. Recarregar a conta com seus pedidos</x:v>
       </x:c>
       <x:c r="G39" s="32" t="str">
-        <x:v>Pedido removido. Pedidos.Count decrementa</x:v>
+        <x:v>Result.IsSuccess. Status=Fechada. Total e snapshots dos pedidos permanecem inalterados</x:v>
       </x:c>
       <x:c r="H39" s="32" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-13, RN-17, RN-19</x:v>
       </x:c>
       <x:c r="I39" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="32" t="str">
-        <x:v>CT39</x:v>
+        <x:v>CT45</x:v>
       </x:c>
       <x:c r="B40" s="32" t="str">
         <x:v>Conta</x:v>
       </x:c>
       <x:c r="C40" s="32" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D40" s="32" t="str">
-        <x:v>Remover pedido em conta fechada lança exceção</x:v>
+        <x:v>Fechar conta com outras contas abertas na mesa</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>Conta fechada com pedidos</x:v>
+        <x:v>Mesa com 2 contas abertas</x:v>
       </x:c>
       <x:c r="F40" s="32" t="str">
-        <x:v>Chamar conta.RemoverPedido(pedidoId)</x:v>
+        <x:v>Chamar Fechar na primeira conta</x:v>
       </x:c>
       <x:c r="G40" s="32" t="str">
-        <x:v>Lança InvalidOperationException</x:v>
+        <x:v>Result.IsSuccess. Conta fechada. Mesa permanece Ocupada (ainda há 1 conta aberta)</x:v>
       </x:c>
       <x:c r="H40" s="32" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-10</x:v>
       </x:c>
       <x:c r="I40" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="24" hidden="0" customHeight="1">
       <x:c r="A41" s="32" t="str">
-        <x:v>CT40</x:v>
+        <x:v>CT46</x:v>
       </x:c>
       <x:c r="B41" s="32" t="str">
         <x:v>Conta</x:v>
@@ -1822,27 +1822,27 @@
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D41" s="32" t="str">
-        <x:v>Abrir conta com dados válidos</x:v>
+        <x:v>Fechar última conta aberta libera mesa</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>Mesa livre, garçom existente, ambos do mesmo UserId</x:v>
+        <x:v>Mesa com 1 conta aberta</x:v>
       </x:c>
       <x:c r="F41" s="32" t="str">
-        <x:v>Chamar Abrir(mesaId, garcomId, "Carlos", userId)</x:v>
+        <x:v>Chamar Fechar(contaId)</x:v>
       </x:c>
       <x:c r="G41" s="32" t="str">
-        <x:v>Result.IsSuccess. Conta persistida. Status=Aberta. DataFechamento=null. Mesa → Ocupada (se era primeira conta)</x:v>
+        <x:v>Result.IsSuccess. Conta fechada. Mesa → Livre (0 contas abertas)</x:v>
       </x:c>
       <x:c r="H41" s="32" t="str">
-        <x:v>RN-01, RN-09, RN-10, RN-12</x:v>
+        <x:v>RN-11</x:v>
       </x:c>
       <x:c r="I41" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="24" hidden="0" customHeight="1">
       <x:c r="A42" s="32" t="str">
-        <x:v>CT41</x:v>
+        <x:v>CT47</x:v>
       </x:c>
       <x:c r="B42" s="32" t="str">
         <x:v>Conta</x:v>
@@ -1851,27 +1851,27 @@
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D42" s="32" t="str">
-        <x:v>Abrir conta em mesa já ocupada</x:v>
+        <x:v>Fechar conta já fechada</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>Mesa ocupada (1 conta aberta existente)</x:v>
+        <x:v>Conta com Status=Fechada</x:v>
       </x:c>
       <x:c r="F42" s="32" t="str">
-        <x:v>Chamar Abrir com a mesma mesa</x:v>
+        <x:v>Chamar Fechar(contaId)</x:v>
       </x:c>
       <x:c r="G42" s="32" t="str">
-        <x:v>Result.IsSuccess. Nova conta criada. Mesa permanece Ocupada. Múltiplas contas abertas permitidas</x:v>
+        <x:v>Result.IsFailed. Erro: "A conta já está fechada."</x:v>
       </x:c>
       <x:c r="H42" s="32" t="str">
-        <x:v>RN-09, RN-10</x:v>
+        <x:v>RN-13</x:v>
       </x:c>
       <x:c r="I42" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="32" t="str">
-        <x:v>CT42</x:v>
+        <x:v>CT48</x:v>
       </x:c>
       <x:c r="B43" s="32" t="str">
         <x:v>Conta</x:v>
@@ -1880,27 +1880,27 @@
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D43" s="32" t="str">
-        <x:v>Abrir conta com mesa de outro usuário</x:v>
+        <x:v>Fechar conta inexistente</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>Mesa pertence a UserId=B, tentar abrir conta com UserId=A</x:v>
+        <x:v>ContaId não existe</x:v>
       </x:c>
       <x:c r="F43" s="32" t="str">
-        <x:v>Chamar Abrir com mesaId de B e userId=A</x:v>
+        <x:v>Chamar Fechar(contaIdInexistente)</x:v>
       </x:c>
       <x:c r="G43" s="32" t="str">
-        <x:v>Result.IsFailed. Erro: "Mesa não encontrada para este usuário."</x:v>
+        <x:v>Result.IsFailed. Erro: "Conta não encontrada."</x:v>
       </x:c>
       <x:c r="H43" s="32" t="str">
-        <x:v>RN-02, RN-12</x:v>
+        <x:v>RN-02</x:v>
       </x:c>
       <x:c r="I43" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
       <x:c r="A44" s="32" t="str">
-        <x:v>CT43</x:v>
+        <x:v>CT49</x:v>
       </x:c>
       <x:c r="B44" s="32" t="str">
         <x:v>Conta</x:v>
@@ -1909,1071 +1909,1071 @@
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D44" s="32" t="str">
-        <x:v>Abrir conta com garçom de outro usuário</x:v>
+        <x:v>Listar contas filtra por UserId</x:v>
       </x:c>
       <x:c r="E44" s="32" t="str">
-        <x:v>Garçom pertence a UserId=B, tentar abrir conta com UserId=A</x:v>
+        <x:v>2 contas: 1 do usuário A, 1 do usuário B</x:v>
       </x:c>
       <x:c r="F44" s="32" t="str">
-        <x:v>Chamar Abrir com garcomId de B e userId=A</x:v>
+        <x:v>Chamar SelecionarTodos() com UserId=A</x:v>
       </x:c>
       <x:c r="G44" s="32" t="str">
-        <x:v>Result.IsFailed. Erro: "Garçom não encontrado para este usuário."</x:v>
+        <x:v>Retorna apenas contas do usuário A</x:v>
       </x:c>
       <x:c r="H44" s="32" t="str">
-        <x:v>RN-02, RN-12</x:v>
+        <x:v>RN-01, RN-02</x:v>
       </x:c>
       <x:c r="I44" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="24" hidden="0" customHeight="1">
       <x:c r="A45" s="32" t="str">
-        <x:v>CT44</x:v>
+        <x:v>CT50</x:v>
       </x:c>
       <x:c r="B45" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C45" s="32" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Domínio</x:v>
       </x:c>
       <x:c r="D45" s="32" t="str">
-        <x:v>Fechar conta preserva total e histórico dos pedidos</x:v>
+        <x:v>Validar pedido com dados válidos</x:v>
       </x:c>
       <x:c r="E45" s="32" t="str">
-        <x:v>Conta aberta com pedidos e produtos posteriormente editados</x:v>
+        <x:v>Nenhuma</x:v>
       </x:c>
       <x:c r="F45" s="32" t="str">
-        <x:v>Registrar o total. Fechar a conta. Recarregar a conta com seus pedidos</x:v>
+        <x:v>Criar pedido com ProdutoId, ProdutoNome="Cerveja", ProdutoPreco=12.00, Quantidade=3. Chamar Validar()</x:v>
       </x:c>
       <x:c r="G45" s="32" t="str">
-        <x:v>Result.IsSuccess. Status=Fechada. Total e snapshots dos pedidos permanecem inalterados</x:v>
+        <x:v>Lista de erros vazia</x:v>
       </x:c>
       <x:c r="H45" s="32" t="str">
-        <x:v>RN-13, RN-17, RN-19</x:v>
+        <x:v>RN-15, RN-17, RN-18</x:v>
       </x:c>
       <x:c r="I45" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="24" hidden="0" customHeight="1">
       <x:c r="A46" s="32" t="str">
-        <x:v>CT45</x:v>
+        <x:v>CT51</x:v>
       </x:c>
       <x:c r="B46" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C46" s="32" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Domínio</x:v>
       </x:c>
       <x:c r="D46" s="32" t="str">
-        <x:v>Fechar conta com outras contas abertas na mesa</x:v>
+        <x:v>Validar pedido com quantidade zero</x:v>
       </x:c>
       <x:c r="E46" s="32" t="str">
-        <x:v>Mesa com 2 contas abertas</x:v>
+        <x:v>Nenhuma</x:v>
       </x:c>
       <x:c r="F46" s="32" t="str">
-        <x:v>Chamar Fechar na primeira conta</x:v>
+        <x:v>Criar pedido com Quantidade=0. Chamar Validar()</x:v>
       </x:c>
       <x:c r="G46" s="32" t="str">
-        <x:v>Result.IsSuccess. Conta fechada. Mesa permanece Ocupada (ainda há 1 conta aberta)</x:v>
+        <x:v>Retorna erro: "O campo Quantidade deve ser maior que zero."</x:v>
       </x:c>
       <x:c r="H46" s="32" t="str">
-        <x:v>RN-10</x:v>
+        <x:v>RN-15</x:v>
       </x:c>
       <x:c r="I46" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="32" t="str">
-        <x:v>CT46</x:v>
+        <x:v>CT52</x:v>
       </x:c>
       <x:c r="B47" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C47" s="32" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Domínio</x:v>
       </x:c>
       <x:c r="D47" s="32" t="str">
-        <x:v>Fechar última conta aberta libera mesa</x:v>
+        <x:v>Validar pedido sem produto</x:v>
       </x:c>
       <x:c r="E47" s="32" t="str">
-        <x:v>Mesa com 1 conta aberta</x:v>
+        <x:v>Nenhuma</x:v>
       </x:c>
       <x:c r="F47" s="32" t="str">
-        <x:v>Chamar Fechar(contaId)</x:v>
+        <x:v>Criar pedido com ProdutoId=Guid.Empty. Chamar Validar()</x:v>
       </x:c>
       <x:c r="G47" s="32" t="str">
-        <x:v>Result.IsSuccess. Conta fechada. Mesa → Livre (0 contas abertas)</x:v>
+        <x:v>Retorna erro: "O campo Produto deve ser selecionado."</x:v>
       </x:c>
       <x:c r="H47" s="32" t="str">
-        <x:v>RN-11</x:v>
+        <x:v>RN-16</x:v>
       </x:c>
       <x:c r="I47" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="32" t="str">
-        <x:v>CT47</x:v>
+        <x:v>CT53</x:v>
       </x:c>
       <x:c r="B48" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C48" s="32" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Domínio</x:v>
       </x:c>
       <x:c r="D48" s="32" t="str">
-        <x:v>Fechar conta já fechada</x:v>
+        <x:v>Subtotal calcula preco x quantidade</x:v>
       </x:c>
       <x:c r="E48" s="32" t="str">
-        <x:v>Conta com Status=Fechada</x:v>
+        <x:v>Pedido com ProdutoPreco=12.00, Quantidade=3</x:v>
       </x:c>
       <x:c r="F48" s="32" t="str">
-        <x:v>Chamar Fechar(contaId)</x:v>
+        <x:v>Verificar pedido.Subtotal</x:v>
       </x:c>
       <x:c r="G48" s="32" t="str">
-        <x:v>Result.IsFailed. Erro: "A conta já está fechada."</x:v>
+        <x:v>Subtotal == 36.00</x:v>
       </x:c>
       <x:c r="H48" s="32" t="str">
-        <x:v>RN-13</x:v>
+        <x:v>RN-18</x:v>
       </x:c>
       <x:c r="I48" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="32" t="str">
-        <x:v>CT48</x:v>
+        <x:v>CT54</x:v>
       </x:c>
       <x:c r="B49" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C49" s="32" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Domínio</x:v>
       </x:c>
       <x:c r="D49" s="32" t="str">
-        <x:v>Fechar conta inexistente</x:v>
+        <x:v>Snapshot preserva nome e preco</x:v>
       </x:c>
       <x:c r="E49" s="32" t="str">
-        <x:v>ContaId não existe</x:v>
+        <x:v>Produto original: Nome="Cerveja", Preco=12</x:v>
       </x:c>
       <x:c r="F49" s="32" t="str">
-        <x:v>Chamar Fechar(contaIdInexistente)</x:v>
+        <x:v>Criar pedido. Alterar produto para Nome="Cerveja Artesanal", Preco=18. Verificar pedido</x:v>
       </x:c>
       <x:c r="G49" s="32" t="str">
-        <x:v>Result.IsFailed. Erro: "Conta não encontrada."</x:v>
+        <x:v>Pedido.ProdutoNome="Cerveja", Pedido.ProdutoPreco=12.00 (inalterado)</x:v>
       </x:c>
       <x:c r="H49" s="32" t="str">
-        <x:v>RN-02</x:v>
+        <x:v>RN-17</x:v>
       </x:c>
       <x:c r="I49" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="32" t="str">
-        <x:v>CT49</x:v>
+        <x:v>CT55</x:v>
       </x:c>
       <x:c r="B50" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C50" s="32" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D50" s="32" t="str">
-        <x:v>Listar contas filtra por UserId</x:v>
+        <x:v>Adicionar pedido em conta aberta</x:v>
       </x:c>
       <x:c r="E50" s="32" t="str">
-        <x:v>2 contas: 1 do usuário A, 1 do usuário B</x:v>
+        <x:v>Conta aberta, produto do mesmo UserId</x:v>
       </x:c>
       <x:c r="F50" s="32" t="str">
-        <x:v>Chamar SelecionarTodos() com UserId=A</x:v>
+        <x:v>Chamar AdicionarPedido(contaId, produtoId, quantidade=2)</x:v>
       </x:c>
       <x:c r="G50" s="32" t="str">
-        <x:v>Retorna apenas contas do usuário A</x:v>
+        <x:v>Result.IsSuccess. Pedido persistido com snapshot de nome e preco</x:v>
       </x:c>
       <x:c r="H50" s="32" t="str">
-        <x:v>RN-01, RN-02</x:v>
+        <x:v>RN-01, RN-16, RN-17</x:v>
       </x:c>
       <x:c r="I50" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="24" hidden="0" customHeight="1">
       <x:c r="A51" s="35" t="str">
-        <x:v>CT50</x:v>
+        <x:v>CT56</x:v>
       </x:c>
       <x:c r="B51" s="35" t="str">
         <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C51" s="35" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D51" s="35" t="str">
-        <x:v>Validar pedido com dados válidos</x:v>
+        <x:v>Adicionar pedido em conta fechada</x:v>
       </x:c>
       <x:c r="E51" s="35" t="str">
-        <x:v>Nenhuma</x:v>
+        <x:v>Conta fechada</x:v>
       </x:c>
       <x:c r="F51" s="35" t="str">
-        <x:v>Criar pedido com ProdutoId, ProdutoNome="Cerveja", ProdutoPreco=12.00, Quantidade=3. Chamar Validar()</x:v>
+        <x:v>Chamar AdicionarPedido(contaId, produtoId, quantidade=2)</x:v>
       </x:c>
       <x:c r="G51" s="35" t="str">
-        <x:v>Lista de erros vazia</x:v>
+        <x:v>Result.IsFailed. Erro: "Não é possível adicionar pedidos a uma conta fechada."</x:v>
       </x:c>
       <x:c r="H51" s="35" t="str">
-        <x:v>RN-15, RN-17, RN-18</x:v>
+        <x:v>RN-14</x:v>
       </x:c>
       <x:c r="I51" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="35" t="str">
-        <x:v>CT51</x:v>
+        <x:v>CT57</x:v>
       </x:c>
       <x:c r="B52" s="35" t="str">
         <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C52" s="35" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D52" s="35" t="str">
-        <x:v>Validar pedido com quantidade zero</x:v>
+        <x:v>Adicionar pedido com produto de outro usuário</x:v>
       </x:c>
       <x:c r="E52" s="35" t="str">
-        <x:v>Nenhuma</x:v>
+        <x:v>Produto pertence a UserId=B, conta pertence a UserId=A</x:v>
       </x:c>
       <x:c r="F52" s="35" t="str">
-        <x:v>Criar pedido com Quantidade=0. Chamar Validar()</x:v>
+        <x:v>Chamar AdicionarPedido com produtoId de B</x:v>
       </x:c>
       <x:c r="G52" s="35" t="str">
-        <x:v>Retorna erro: "O campo Quantidade deve ser maior que zero."</x:v>
+        <x:v>Result.IsFailed. Erro: "Produto não encontrado para este usuário."</x:v>
       </x:c>
       <x:c r="H52" s="35" t="str">
-        <x:v>RN-15</x:v>
+        <x:v>RN-02, RN-16</x:v>
       </x:c>
       <x:c r="I52" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="35" t="str">
-        <x:v>CT52</x:v>
+        <x:v>CT58</x:v>
       </x:c>
       <x:c r="B53" s="35" t="str">
         <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C53" s="35" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D53" s="35" t="str">
-        <x:v>Validar pedido sem produto</x:v>
+        <x:v>Adicionar pedido com quantidade zero</x:v>
       </x:c>
       <x:c r="E53" s="35" t="str">
-        <x:v>Nenhuma</x:v>
+        <x:v>Conta aberta</x:v>
       </x:c>
       <x:c r="F53" s="35" t="str">
-        <x:v>Criar pedido com ProdutoId=Guid.Empty. Chamar Validar()</x:v>
+        <x:v>Chamar AdicionarPedido com quantidade=0</x:v>
       </x:c>
       <x:c r="G53" s="35" t="str">
-        <x:v>Retorna erro: "O campo Produto deve ser selecionado."</x:v>
+        <x:v>Result.IsFailed. Erro: "A quantidade deve ser maior que zero."</x:v>
       </x:c>
       <x:c r="H53" s="35" t="str">
-        <x:v>RN-16</x:v>
+        <x:v>RN-15</x:v>
       </x:c>
       <x:c r="I53" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="24" hidden="0" customHeight="1">
       <x:c r="A54" s="35" t="str">
-        <x:v>CT53</x:v>
+        <x:v>CT59</x:v>
       </x:c>
       <x:c r="B54" s="35" t="str">
         <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C54" s="35" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D54" s="35" t="str">
-        <x:v>Subtotal calcula preco x quantidade</x:v>
+        <x:v>Remover pedido de conta aberta</x:v>
       </x:c>
       <x:c r="E54" s="35" t="str">
-        <x:v>Pedido com ProdutoPreco=12.00, Quantidade=3</x:v>
+        <x:v>Conta aberta com 1 pedido</x:v>
       </x:c>
       <x:c r="F54" s="35" t="str">
-        <x:v>Verificar pedido.Subtotal</x:v>
+        <x:v>Chamar RemoverPedido(contaId, pedidoId)</x:v>
       </x:c>
       <x:c r="G54" s="35" t="str">
-        <x:v>Subtotal == 36.00</x:v>
+        <x:v>Result.IsSuccess. Pedido removido da conta</x:v>
       </x:c>
       <x:c r="H54" s="35" t="str">
-        <x:v>RN-18</x:v>
+        <x:v>RN-14</x:v>
       </x:c>
       <x:c r="I54" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="24" hidden="0" customHeight="1">
       <x:c r="A55" s="35" t="str">
-        <x:v>CT54</x:v>
+        <x:v>CT60</x:v>
       </x:c>
       <x:c r="B55" s="35" t="str">
         <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C55" s="35" t="str">
-        <x:v>Domínio</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D55" s="35" t="str">
-        <x:v>Snapshot preserva nome e preco</x:v>
+        <x:v>Remover pedido de conta fechada</x:v>
       </x:c>
       <x:c r="E55" s="35" t="str">
-        <x:v>Produto original: Nome="Cerveja", Preco=12</x:v>
+        <x:v>Conta fechada com pedidos</x:v>
       </x:c>
       <x:c r="F55" s="35" t="str">
-        <x:v>Criar pedido. Alterar produto para Nome="Cerveja Artesanal", Preco=18. Verificar pedido</x:v>
+        <x:v>Chamar RemoverPedido(contaId, pedidoId)</x:v>
       </x:c>
       <x:c r="G55" s="35" t="str">
-        <x:v>Pedido.ProdutoNome="Cerveja", Pedido.ProdutoPreco=12.00 (inalterado)</x:v>
+        <x:v>Result.IsFailed. Erro: "Não é possível remover pedidos de uma conta fechada."</x:v>
       </x:c>
       <x:c r="H55" s="35" t="str">
-        <x:v>RN-17</x:v>
+        <x:v>RN-14</x:v>
       </x:c>
       <x:c r="I55" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="24" hidden="0" customHeight="1">
       <x:c r="A56" s="35" t="str">
-        <x:v>CT55</x:v>
+        <x:v>CT61</x:v>
       </x:c>
       <x:c r="B56" s="35" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Faturamento</x:v>
       </x:c>
       <x:c r="C56" s="35" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D56" s="35" t="str">
-        <x:v>Adicionar pedido em conta aberta</x:v>
+        <x:v>Calcular faturamento diário com contas fechadas</x:v>
       </x:c>
       <x:c r="E56" s="35" t="str">
-        <x:v>Conta aberta, produto do mesmo UserId</x:v>
+        <x:v>3 contas fechadas hoje: R$50, R$30, R$20</x:v>
       </x:c>
       <x:c r="F56" s="35" t="str">
-        <x:v>Chamar AdicionarPedido(contaId, produtoId, quantidade=2)</x:v>
+        <x:v>Chamar CalcularFaturamento(dataHoje, userId)</x:v>
       </x:c>
       <x:c r="G56" s="35" t="str">
-        <x:v>Result.IsSuccess. Pedido persistido com snapshot de nome e preco</x:v>
+        <x:v>Retorna R$100.00</x:v>
       </x:c>
       <x:c r="H56" s="35" t="str">
-        <x:v>RN-01, RN-16, RN-17</x:v>
+        <x:v>RN-20</x:v>
       </x:c>
       <x:c r="I56" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="24" hidden="0" customHeight="1">
       <x:c r="A57" s="35" t="str">
-        <x:v>CT56</x:v>
+        <x:v>CT62</x:v>
       </x:c>
       <x:c r="B57" s="35" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Faturamento</x:v>
       </x:c>
       <x:c r="C57" s="35" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D57" s="35" t="str">
-        <x:v>Adicionar pedido em conta fechada</x:v>
+        <x:v>Faturamento ignora contas abertas</x:v>
       </x:c>
       <x:c r="E57" s="35" t="str">
-        <x:v>Conta fechada</x:v>
+        <x:v>2 contas: 1 aberta R$50, 1 fechada R$30 (hoje)</x:v>
       </x:c>
       <x:c r="F57" s="35" t="str">
-        <x:v>Chamar AdicionarPedido(contaId, produtoId, quantidade=2)</x:v>
+        <x:v>Chamar CalcularFaturamento(dataHoje, userId)</x:v>
       </x:c>
       <x:c r="G57" s="35" t="str">
-        <x:v>Result.IsFailed. Erro: "Não é possível adicionar pedidos a uma conta fechada."</x:v>
+        <x:v>Retorna R$30.00 (apenas fechada)</x:v>
       </x:c>
       <x:c r="H57" s="35" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-20</x:v>
       </x:c>
       <x:c r="I57" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="24" hidden="0" customHeight="1">
       <x:c r="A58" s="35" t="str">
-        <x:v>CT57</x:v>
+        <x:v>CT63</x:v>
       </x:c>
       <x:c r="B58" s="35" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Faturamento</x:v>
       </x:c>
       <x:c r="C58" s="35" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D58" s="35" t="str">
-        <x:v>Adicionar pedido com produto de outro usuário</x:v>
+        <x:v>Faturamento ignora contas de outros dias</x:v>
       </x:c>
       <x:c r="E58" s="35" t="str">
-        <x:v>Produto pertence a UserId=B, conta pertence a UserId=A</x:v>
+        <x:v>1 conta fechada hoje R$50, 1 conta fechada ontem R$100</x:v>
       </x:c>
       <x:c r="F58" s="35" t="str">
-        <x:v>Chamar AdicionarPedido com produtoId de B</x:v>
+        <x:v>Chamar CalcularFaturamento(dataHoje, userId)</x:v>
       </x:c>
       <x:c r="G58" s="35" t="str">
-        <x:v>Result.IsFailed. Erro: "Produto não encontrado para este usuário."</x:v>
+        <x:v>Retorna R$50.00</x:v>
       </x:c>
       <x:c r="H58" s="35" t="str">
-        <x:v>RN-02, RN-16</x:v>
+        <x:v>RN-20</x:v>
       </x:c>
       <x:c r="I58" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="35" t="str">
-        <x:v>CT58</x:v>
+        <x:v>CT64</x:v>
       </x:c>
       <x:c r="B59" s="35" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Faturamento</x:v>
       </x:c>
       <x:c r="C59" s="35" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D59" s="35" t="str">
-        <x:v>Adicionar pedido com quantidade zero</x:v>
+        <x:v>Faturamento filtra por UserId</x:v>
       </x:c>
       <x:c r="E59" s="35" t="str">
-        <x:v>Conta aberta</x:v>
+        <x:v>Conta fechada hoje do usuário A R$50, conta fechada hoje do usuário B R$100</x:v>
       </x:c>
       <x:c r="F59" s="35" t="str">
-        <x:v>Chamar AdicionarPedido com quantidade=0</x:v>
+        <x:v>Chamar CalcularFaturamento(dataHoje, userId=A)</x:v>
       </x:c>
       <x:c r="G59" s="35" t="str">
-        <x:v>Result.IsFailed. Erro: "A quantidade deve ser maior que zero."</x:v>
+        <x:v>Retorna R$50.00</x:v>
       </x:c>
       <x:c r="H59" s="35" t="str">
-        <x:v>RN-15</x:v>
+        <x:v>RN-01, RN-02, RN-20</x:v>
       </x:c>
       <x:c r="I59" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="35" t="str">
-        <x:v>CT59</x:v>
+        <x:v>CT65</x:v>
       </x:c>
       <x:c r="B60" s="35" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Faturamento</x:v>
       </x:c>
       <x:c r="C60" s="35" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D60" s="35" t="str">
-        <x:v>Remover pedido de conta aberta</x:v>
+        <x:v>Faturamento de dia sem contas fechadas</x:v>
       </x:c>
       <x:c r="E60" s="35" t="str">
-        <x:v>Conta aberta com 1 pedido</x:v>
+        <x:v>Nenhuma conta fechada na data</x:v>
       </x:c>
       <x:c r="F60" s="35" t="str">
-        <x:v>Chamar RemoverPedido(contaId, pedidoId)</x:v>
+        <x:v>Chamar CalcularFaturamento(dataSemContas, userId)</x:v>
       </x:c>
       <x:c r="G60" s="35" t="str">
-        <x:v>Result.IsSuccess. Pedido removido da conta</x:v>
+        <x:v>Retorna R$0.00</x:v>
       </x:c>
       <x:c r="H60" s="35" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-20</x:v>
       </x:c>
       <x:c r="I60" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="24" hidden="0" customHeight="1">
       <x:c r="A61" s="35" t="str">
-        <x:v>CT60</x:v>
+        <x:v>CT66</x:v>
       </x:c>
       <x:c r="B61" s="35" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Autenticação</x:v>
       </x:c>
       <x:c r="C61" s="35" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D61" s="35" t="str">
-        <x:v>Remover pedido de conta fechada</x:v>
+        <x:v>Registrar novo usuário</x:v>
       </x:c>
       <x:c r="E61" s="35" t="str">
-        <x:v>Conta fechada com pedidos</x:v>
+        <x:v>Nenhuma</x:v>
       </x:c>
       <x:c r="F61" s="35" t="str">
-        <x:v>Chamar RemoverPedido(contaId, pedidoId)</x:v>
+        <x:v>Preencher e-mail e senha. Clicar Registrar</x:v>
       </x:c>
       <x:c r="G61" s="35" t="str">
-        <x:v>Result.IsFailed. Erro: "Não é possível remover pedidos de uma conta fechada."</x:v>
+        <x:v>Usuário criado. Login automático. Redireciona para Dashboard</x:v>
       </x:c>
       <x:c r="H61" s="35" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>Funcionalidade: Autenticação</x:v>
       </x:c>
       <x:c r="I61" s="35" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="38" t="str">
-        <x:v>CT61</x:v>
+        <x:v>CT67</x:v>
       </x:c>
       <x:c r="B62" s="38" t="str">
-        <x:v>Faturamento</x:v>
+        <x:v>Autenticação</x:v>
       </x:c>
       <x:c r="C62" s="38" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D62" s="38" t="str">
-        <x:v>Calcular faturamento diário com contas fechadas</x:v>
+        <x:v>Login com credenciais válidas</x:v>
       </x:c>
       <x:c r="E62" s="38" t="str">
-        <x:v>3 contas fechadas hoje: R$50, R$30, R$20</x:v>
+        <x:v>Usuário registrado</x:v>
       </x:c>
       <x:c r="F62" s="38" t="str">
-        <x:v>Chamar CalcularFaturamento(dataHoje, userId)</x:v>
+        <x:v>Inserir e-mail e senha. Clicar Entrar</x:v>
       </x:c>
       <x:c r="G62" s="38" t="str">
-        <x:v>Retorna R$100.00</x:v>
+        <x:v>Autenticação bem-sucedida. Redireciona para Dashboard</x:v>
       </x:c>
       <x:c r="H62" s="38" t="str">
-        <x:v>RN-20</x:v>
+        <x:v>Funcionalidade: Autenticação</x:v>
       </x:c>
       <x:c r="I62" s="38" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="24" hidden="0" customHeight="1">
       <x:c r="A63" s="38" t="str">
-        <x:v>CT62</x:v>
+        <x:v>CT68</x:v>
       </x:c>
       <x:c r="B63" s="38" t="str">
-        <x:v>Faturamento</x:v>
+        <x:v>Autenticação</x:v>
       </x:c>
       <x:c r="C63" s="38" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D63" s="38" t="str">
-        <x:v>Faturamento ignora contas abertas</x:v>
+        <x:v>Login com senha inválida</x:v>
       </x:c>
       <x:c r="E63" s="38" t="str">
-        <x:v>2 contas: 1 aberta R$50, 1 fechada R$30 (hoje)</x:v>
+        <x:v>Usuário registrado</x:v>
       </x:c>
       <x:c r="F63" s="38" t="str">
-        <x:v>Chamar CalcularFaturamento(dataHoje, userId)</x:v>
+        <x:v>Inserir e-mail correto e senha errada. Clicar Entrar</x:v>
       </x:c>
       <x:c r="G63" s="38" t="str">
-        <x:v>Retorna R$30.00 (apenas fechada)</x:v>
+        <x:v>Mensagem de erro. Permanece na tela de login</x:v>
       </x:c>
       <x:c r="H63" s="38" t="str">
-        <x:v>RN-20</x:v>
+        <x:v>Funcionalidade: Autenticação</x:v>
       </x:c>
       <x:c r="I63" s="38" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="24" hidden="0" customHeight="1">
       <x:c r="A64" s="38" t="str">
-        <x:v>CT63</x:v>
+        <x:v>CT69</x:v>
       </x:c>
       <x:c r="B64" s="38" t="str">
-        <x:v>Faturamento</x:v>
+        <x:v>Autenticação</x:v>
       </x:c>
       <x:c r="C64" s="38" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D64" s="38" t="str">
-        <x:v>Faturamento ignora contas de outros dias</x:v>
+        <x:v>Acesso sem login redireciona</x:v>
       </x:c>
       <x:c r="E64" s="38" t="str">
-        <x:v>1 conta fechada hoje R$50, 1 conta fechada ontem R$100</x:v>
+        <x:v>Usuário não autenticado</x:v>
       </x:c>
       <x:c r="F64" s="38" t="str">
-        <x:v>Chamar CalcularFaturamento(dataHoje, userId)</x:v>
+        <x:v>Acessar /Mesas diretamente</x:v>
       </x:c>
       <x:c r="G64" s="38" t="str">
-        <x:v>Retorna R$50.00</x:v>
+        <x:v>Redireciona para a tela de entrada da aplicação</x:v>
       </x:c>
       <x:c r="H64" s="38" t="str">
-        <x:v>RN-20</x:v>
+        <x:v>Funcionalidade: Autenticação</x:v>
       </x:c>
       <x:c r="I64" s="38" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="24" hidden="0" customHeight="1">
       <x:c r="A65" s="38" t="str">
-        <x:v>CT64</x:v>
+        <x:v>CT70</x:v>
       </x:c>
       <x:c r="B65" s="38" t="str">
-        <x:v>Faturamento</x:v>
+        <x:v>Autenticação</x:v>
       </x:c>
       <x:c r="C65" s="38" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D65" s="38" t="str">
-        <x:v>Faturamento filtra por UserId</x:v>
+        <x:v>Logout</x:v>
       </x:c>
       <x:c r="E65" s="38" t="str">
-        <x:v>Conta fechada hoje do usuário A R$50, conta fechada hoje do usuário B R$100</x:v>
+        <x:v>Usuário logado</x:v>
       </x:c>
       <x:c r="F65" s="38" t="str">
-        <x:v>Chamar CalcularFaturamento(dataHoje, userId=A)</x:v>
+        <x:v>Clicar Sair</x:v>
       </x:c>
       <x:c r="G65" s="38" t="str">
-        <x:v>Retorna R$50.00</x:v>
+        <x:v>Sessão encerrada. Redireciona para /Login</x:v>
       </x:c>
       <x:c r="H65" s="38" t="str">
-        <x:v>RN-01, RN-02, RN-20</x:v>
+        <x:v>Funcionalidade: Autenticação</x:v>
       </x:c>
       <x:c r="I65" s="38" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="38" t="str">
-        <x:v>CT65</x:v>
+        <x:v>CT71</x:v>
       </x:c>
       <x:c r="B66" s="38" t="str">
-        <x:v>Faturamento</x:v>
+        <x:v>Conta</x:v>
       </x:c>
       <x:c r="C66" s="38" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D66" s="38" t="str">
-        <x:v>Faturamento de dia sem contas fechadas</x:v>
+        <x:v>Fluxo completo: abrir conta, adicionar pedidos, fechar</x:v>
       </x:c>
       <x:c r="E66" s="38" t="str">
-        <x:v>Nenhuma conta fechada na data</x:v>
+        <x:v>Usuário logado. Mesa, garçom e produto cadastrados</x:v>
       </x:c>
       <x:c r="F66" s="38" t="str">
-        <x:v>Chamar CalcularFaturamento(dataSemContas, userId)</x:v>
+        <x:v>1. Abrir conta na mesa. 2. Adicionar 2 pedidos. 3. Verificar total. 4. Fechar conta. 5. Verificar mesa livre</x:v>
       </x:c>
       <x:c r="G66" s="38" t="str">
-        <x:v>Retorna R$0.00</x:v>
+        <x:v>Conta criada. Pedidos adicionados. Total correto. Conta fechada. Mesa volta para Livre</x:v>
       </x:c>
       <x:c r="H66" s="38" t="str">
-        <x:v>RN-20</x:v>
+        <x:v>RN-09, RN-10, RN-11, RN-14, RN-19</x:v>
       </x:c>
       <x:c r="I66" s="38" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="24" hidden="0" customHeight="1">
       <x:c r="A67" s="41" t="str">
-        <x:v>CT66</x:v>
+        <x:v>CT72</x:v>
       </x:c>
       <x:c r="B67" s="41" t="str">
-        <x:v>Autenticação</x:v>
+        <x:v>Conta</x:v>
       </x:c>
       <x:c r="C67" s="41" t="str">
         <x:v>E2E</x:v>
       </x:c>
       <x:c r="D67" s="41" t="str">
-        <x:v>Registrar novo usuário</x:v>
+        <x:v>Múltiplas contas na mesma mesa</x:v>
       </x:c>
       <x:c r="E67" s="41" t="str">
-        <x:v>Nenhuma</x:v>
+        <x:v>Usuário logado. Mesa e garçom cadastrados</x:v>
       </x:c>
       <x:c r="F67" s="41" t="str">
-        <x:v>Preencher e-mail e senha. Clicar Registrar</x:v>
+        <x:v>1. Abrir conta A na mesa 1. 2. Abrir conta B na mesma mesa. 3. Fechar conta A. 4. Verificar mesa ocupada. 5. Fechar conta B. 6. Verificar mesa livre</x:v>
       </x:c>
       <x:c r="G67" s="41" t="str">
-        <x:v>Usuário criado. Login automático. Redireciona para Dashboard</x:v>
+        <x:v>Mesa permite 2 contas abertas. Ao fechar A, mesa permanece ocupada. Ao fechar B, mesa fica livre</x:v>
       </x:c>
       <x:c r="H67" s="41" t="str">
-        <x:v>Funcionalidade: Autenticação</x:v>
+        <x:v>RN-09, RN-10, RN-11</x:v>
       </x:c>
       <x:c r="I67" s="41" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="24" hidden="0" customHeight="1">
       <x:c r="A68" s="41" t="str">
-        <x:v>CT67</x:v>
+        <x:v>CT73</x:v>
       </x:c>
       <x:c r="B68" s="41" t="str">
-        <x:v>Autenticação</x:v>
+        <x:v>Conta</x:v>
       </x:c>
       <x:c r="C68" s="41" t="str">
         <x:v>E2E</x:v>
       </x:c>
       <x:c r="D68" s="41" t="str">
-        <x:v>Login com credenciais válidas</x:v>
+        <x:v>Snapshot de produto preservado após edição</x:v>
       </x:c>
       <x:c r="E68" s="41" t="str">
-        <x:v>Usuário registrado</x:v>
+        <x:v>Usuário logado. Produto "Cerveja" R$12 cadastrado</x:v>
       </x:c>
       <x:c r="F68" s="41" t="str">
-        <x:v>Inserir e-mail e senha. Clicar Entrar</x:v>
+        <x:v>1. Abrir conta. 2. Adicionar pedido (Cerveja x2). 3. Editar produto para R$18. 4. Verificar pedido na conta</x:v>
       </x:c>
       <x:c r="G68" s="41" t="str">
-        <x:v>Autenticação bem-sucedida. Redireciona para Dashboard</x:v>
+        <x:v>Pedido mantém ProdutoPreco=12.00. Valor da conta não muda</x:v>
       </x:c>
       <x:c r="H68" s="41" t="str">
-        <x:v>Funcionalidade: Autenticação</x:v>
+        <x:v>RN-17, RN-19</x:v>
       </x:c>
       <x:c r="I68" s="41" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="24" hidden="0" customHeight="1">
       <x:c r="A69" s="41" t="str">
-        <x:v>CT68</x:v>
+        <x:v>CT74</x:v>
       </x:c>
       <x:c r="B69" s="41" t="str">
-        <x:v>Autenticação</x:v>
+        <x:v>Conta</x:v>
       </x:c>
       <x:c r="C69" s="41" t="str">
         <x:v>E2E</x:v>
       </x:c>
       <x:c r="D69" s="41" t="str">
-        <x:v>Login com senha inválida</x:v>
+        <x:v>Tentar adicionar pedido em conta fechada</x:v>
       </x:c>
       <x:c r="E69" s="41" t="str">
-        <x:v>Usuário registrado</x:v>
+        <x:v>Usuário logado. Mesa, garçom e produto cadastrados</x:v>
       </x:c>
       <x:c r="F69" s="41" t="str">
-        <x:v>Inserir e-mail correto e senha errada. Clicar Entrar</x:v>
+        <x:v>1. Abrir conta. 2. Fechar conta. 3. Acessar seus detalhes. 4. Tentar adicionar pedido</x:v>
       </x:c>
       <x:c r="G69" s="41" t="str">
-        <x:v>Mensagem de erro. Permanece na tela de login</x:v>
+        <x:v>Botão/mensagem indica que não é possível adicionar pedidos a conta fechada</x:v>
       </x:c>
       <x:c r="H69" s="41" t="str">
-        <x:v>Funcionalidade: Autenticação</x:v>
+        <x:v>RN-14</x:v>
       </x:c>
       <x:c r="I69" s="41" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="24" hidden="0" customHeight="1">
       <x:c r="A70" s="41" t="str">
-        <x:v>CT69</x:v>
+        <x:v>CT75</x:v>
       </x:c>
       <x:c r="B70" s="41" t="str">
-        <x:v>Autenticação</x:v>
+        <x:v>Faturamento</x:v>
       </x:c>
       <x:c r="C70" s="41" t="str">
         <x:v>E2E</x:v>
       </x:c>
       <x:c r="D70" s="41" t="str">
-        <x:v>Acesso sem login redireciona</x:v>
+        <x:v>Faturamento diário exibe contas fechadas</x:v>
       </x:c>
       <x:c r="E70" s="41" t="str">
-        <x:v>Usuário não autenticado</x:v>
+        <x:v>Usuário logado. Contas fechadas hoje</x:v>
       </x:c>
       <x:c r="F70" s="41" t="str">
-        <x:v>Acessar /Mesas diretamente</x:v>
+        <x:v>1. Abrir Dashboard. 2. Navegar para Faturamento. 3. Selecionar data de hoje</x:v>
       </x:c>
       <x:c r="G70" s="41" t="str">
-        <x:v>Redireciona para a tela de entrada da aplicação</x:v>
+        <x:v>Card mostra total correto. Tabela lista contas fechadas com valor e horário</x:v>
       </x:c>
       <x:c r="H70" s="41" t="str">
-        <x:v>Funcionalidade: Autenticação</x:v>
+        <x:v>RN-20</x:v>
       </x:c>
       <x:c r="I70" s="41" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="24" hidden="0" customHeight="1">
       <x:c r="A71" s="41" t="str">
-        <x:v>CT70</x:v>
+        <x:v>CT76</x:v>
       </x:c>
       <x:c r="B71" s="41" t="str">
-        <x:v>Autenticação</x:v>
+        <x:v>Mesa</x:v>
       </x:c>
       <x:c r="C71" s="41" t="str">
-        <x:v>E2E</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D71" s="41" t="str">
-        <x:v>Logout</x:v>
+        <x:v>Editar mesa para número já utilizado</x:v>
       </x:c>
       <x:c r="E71" s="41" t="str">
-        <x:v>Usuário logado</x:v>
+        <x:v>Duas mesas do mesmo usuário, números 1 e 2</x:v>
       </x:c>
       <x:c r="F71" s="41" t="str">
-        <x:v>Clicar Sair</x:v>
+        <x:v>Editar a mesa 2 informando Numero=1</x:v>
       </x:c>
       <x:c r="G71" s="41" t="str">
-        <x:v>Sessão encerrada. Redireciona para /Login</x:v>
+        <x:v>Result.IsFailed. A alteração não é persistida</x:v>
       </x:c>
       <x:c r="H71" s="41" t="str">
-        <x:v>Funcionalidade: Autenticação</x:v>
+        <x:v>RN-03</x:v>
       </x:c>
       <x:c r="I71" s="41" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="36" hidden="0" customHeight="1">
       <x:c r="A72" s="32" t="str">
-        <x:v>CT71</x:v>
+        <x:v>CT77</x:v>
       </x:c>
       <x:c r="B72" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Garçom</x:v>
       </x:c>
       <x:c r="C72" s="32" t="str">
-        <x:v>E2E</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D72" s="32" t="str">
-        <x:v>Fluxo completo: abrir conta, adicionar pedidos, fechar</x:v>
+        <x:v>Editar garçom para nome já utilizado</x:v>
       </x:c>
       <x:c r="E72" s="32" t="str">
-        <x:v>Usuário logado. Mesa, garçom e produto cadastrados</x:v>
+        <x:v>Garçons João e Maria do mesmo usuário</x:v>
       </x:c>
       <x:c r="F72" s="32" t="str">
-        <x:v>1. Abrir conta na mesa. 2. Adicionar 2 pedidos. 3. Verificar total. 4. Fechar conta. 5. Verificar mesa livre</x:v>
+        <x:v>Editar Maria informando Nome="João"</x:v>
       </x:c>
       <x:c r="G72" s="32" t="str">
-        <x:v>Conta criada. Pedidos adicionados. Total correto. Conta fechada. Mesa volta para Livre</x:v>
+        <x:v>Result.IsFailed. A alteração não é persistida</x:v>
       </x:c>
       <x:c r="H72" s="32" t="str">
-        <x:v>RN-09, RN-10, RN-11, RN-14, RN-19</x:v>
+        <x:v>RN-05</x:v>
       </x:c>
       <x:c r="I72" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="36" hidden="0" customHeight="1">
       <x:c r="A73" s="32" t="str">
-        <x:v>CT72</x:v>
+        <x:v>CT78</x:v>
       </x:c>
       <x:c r="B73" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Produto</x:v>
       </x:c>
       <x:c r="C73" s="32" t="str">
-        <x:v>E2E</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D73" s="32" t="str">
-        <x:v>Múltiplas contas na mesma mesa</x:v>
+        <x:v>Editar produto para nome já utilizado</x:v>
       </x:c>
       <x:c r="E73" s="32" t="str">
-        <x:v>Usuário logado. Mesa e garçom cadastrados</x:v>
+        <x:v>Produtos Cerveja e Água do mesmo usuário</x:v>
       </x:c>
       <x:c r="F73" s="32" t="str">
-        <x:v>1. Abrir conta A na mesa 1. 2. Abrir conta B na mesma mesa. 3. Fechar conta A. 4. Verificar mesa ocupada. 5. Fechar conta B. 6. Verificar mesa livre</x:v>
+        <x:v>Editar Água informando Nome="Cerveja"</x:v>
       </x:c>
       <x:c r="G73" s="32" t="str">
-        <x:v>Mesa permite 2 contas abertas. Ao fechar A, mesa permanece ocupada. Ao fechar B, mesa fica livre</x:v>
+        <x:v>Result.IsFailed. A alteração não é persistida</x:v>
       </x:c>
       <x:c r="H73" s="32" t="str">
-        <x:v>RN-09, RN-10, RN-11</x:v>
+        <x:v>RN-06</x:v>
       </x:c>
       <x:c r="I73" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="24" hidden="0" customHeight="1">
       <x:c r="A74" s="32" t="str">
-        <x:v>CT73</x:v>
+        <x:v>CT79</x:v>
       </x:c>
       <x:c r="B74" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Mesa</x:v>
       </x:c>
       <x:c r="C74" s="32" t="str">
-        <x:v>E2E</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D74" s="32" t="str">
-        <x:v>Snapshot de produto preservado após edição</x:v>
+        <x:v>Editar mesa de outro usuário</x:v>
       </x:c>
       <x:c r="E74" s="32" t="str">
-        <x:v>Usuário logado. Produto "Cerveja" R$12 cadastrado</x:v>
+        <x:v>Mesa pertence ao usuário B</x:v>
       </x:c>
       <x:c r="F74" s="32" t="str">
-        <x:v>1. Abrir conta. 2. Adicionar pedido (Cerveja x2). 3. Editar produto para R$18. 4. Verificar pedido na conta</x:v>
+        <x:v>Usuário A tenta editar a mesa de B</x:v>
       </x:c>
       <x:c r="G74" s="32" t="str">
-        <x:v>Pedido mantém ProdutoPreco=12.00. Valor da conta não muda</x:v>
+        <x:v>Result.IsFailed. Registro não é alterado</x:v>
       </x:c>
       <x:c r="H74" s="32" t="str">
-        <x:v>RN-17, RN-19</x:v>
+        <x:v>RN-02</x:v>
       </x:c>
       <x:c r="I74" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="24" hidden="0" customHeight="1">
       <x:c r="A75" s="32" t="str">
-        <x:v>CT74</x:v>
+        <x:v>CT80</x:v>
       </x:c>
       <x:c r="B75" s="32" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Garçom</x:v>
       </x:c>
       <x:c r="C75" s="32" t="str">
-        <x:v>E2E</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D75" s="32" t="str">
-        <x:v>Tentar adicionar pedido em conta fechada</x:v>
+        <x:v>Excluir garçom de outro usuário</x:v>
       </x:c>
       <x:c r="E75" s="32" t="str">
-        <x:v>Usuário logado. Mesa, garçom e produto cadastrados</x:v>
+        <x:v>Garçom pertence ao usuário B</x:v>
       </x:c>
       <x:c r="F75" s="32" t="str">
-        <x:v>1. Abrir conta. 2. Fechar conta. 3. Acessar seus detalhes. 4. Tentar adicionar pedido</x:v>
+        <x:v>Usuário A tenta excluir o garçom de B</x:v>
       </x:c>
       <x:c r="G75" s="32" t="str">
-        <x:v>Botão/mensagem indica que não é possível adicionar pedidos a conta fechada</x:v>
+        <x:v>Result.IsFailed. Registro permanece persistido</x:v>
       </x:c>
       <x:c r="H75" s="32" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-02</x:v>
       </x:c>
       <x:c r="I75" s="32" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="24" hidden="0" customHeight="1">
       <x:c r="A76" s="38" t="str">
-        <x:v>CT75</x:v>
+        <x:v>CT81</x:v>
       </x:c>
       <x:c r="B76" s="38" t="str">
-        <x:v>Faturamento</x:v>
+        <x:v>Produto</x:v>
       </x:c>
       <x:c r="C76" s="38" t="str">
-        <x:v>E2E</x:v>
+        <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D76" s="38" t="str">
-        <x:v>Faturamento diário exibe contas fechadas</x:v>
+        <x:v>Excluir produto de outro usuário</x:v>
       </x:c>
       <x:c r="E76" s="38" t="str">
-        <x:v>Usuário logado. Contas fechadas hoje</x:v>
+        <x:v>Produto pertence ao usuário B</x:v>
       </x:c>
       <x:c r="F76" s="38" t="str">
-        <x:v>1. Abrir Dashboard. 2. Navegar para Faturamento. 3. Selecionar data de hoje</x:v>
+        <x:v>Usuário A tenta excluir o produto de B</x:v>
       </x:c>
       <x:c r="G76" s="38" t="str">
-        <x:v>Card mostra total correto. Tabela lista contas fechadas com valor e horário</x:v>
+        <x:v>Result.IsFailed. Registro permanece persistido</x:v>
       </x:c>
       <x:c r="H76" s="38" t="str">
-        <x:v>RN-20</x:v>
+        <x:v>RN-02</x:v>
       </x:c>
       <x:c r="I76" s="38" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
       <x:c r="A77" s="15" t="str">
-        <x:v>CT76</x:v>
+        <x:v>CT82</x:v>
       </x:c>
       <x:c r="B77" s="15" t="str">
-        <x:v>Mesa</x:v>
+        <x:v>Conta</x:v>
       </x:c>
       <x:c r="C77" s="15" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D77" s="15" t="str">
-        <x:v>Editar mesa para número já utilizado</x:v>
+        <x:v>Fechar conta de outro usuário</x:v>
       </x:c>
       <x:c r="E77" s="15" t="str">
-        <x:v>Duas mesas do mesmo usuário, números 1 e 2</x:v>
+        <x:v>Conta pertence ao usuário B</x:v>
       </x:c>
       <x:c r="F77" s="15" t="str">
-        <x:v>Editar a mesa 2 informando Numero=1</x:v>
+        <x:v>Usuário A tenta fechar a conta de B</x:v>
       </x:c>
       <x:c r="G77" s="15" t="str">
-        <x:v>Result.IsFailed. A alteração não é persistida</x:v>
+        <x:v>Result.IsFailed. Conta permanece aberta</x:v>
       </x:c>
       <x:c r="H77" s="15" t="str">
-        <x:v>RN-03</x:v>
+        <x:v>RN-02</x:v>
       </x:c>
       <x:c r="I77" s="15" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
       <x:c r="A78" s="22" t="str">
-        <x:v>CT77</x:v>
+        <x:v>CT83</x:v>
       </x:c>
       <x:c r="B78" s="22" t="str">
-        <x:v>Garçom</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C78" s="22" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D78" s="22" t="str">
-        <x:v>Editar garçom para nome já utilizado</x:v>
+        <x:v>Adicionar pedido em conta inexistente</x:v>
       </x:c>
       <x:c r="E78" s="22" t="str">
-        <x:v>Garçons João e Maria do mesmo usuário</x:v>
+        <x:v>Produto válido do usuário</x:v>
       </x:c>
       <x:c r="F78" s="22" t="str">
-        <x:v>Editar Maria informando Nome="João"</x:v>
+        <x:v>Adicionar pedido usando ContaId inexistente</x:v>
       </x:c>
       <x:c r="G78" s="22" t="str">
-        <x:v>Result.IsFailed. A alteração não é persistida</x:v>
+        <x:v>Result.IsFailed. Nenhum pedido é persistido</x:v>
       </x:c>
       <x:c r="H78" s="22" t="str">
-        <x:v>RN-05</x:v>
+        <x:v>RN-02</x:v>
       </x:c>
       <x:c r="I78" s="22" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
       <x:c r="A79" s="29" t="str">
-        <x:v>CT78</x:v>
+        <x:v>CT84</x:v>
       </x:c>
       <x:c r="B79" s="29" t="str">
-        <x:v>Produto</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C79" s="29" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D79" s="29" t="str">
-        <x:v>Editar produto para nome já utilizado</x:v>
+        <x:v>Adicionar pedido com produto inexistente</x:v>
       </x:c>
       <x:c r="E79" s="29" t="str">
-        <x:v>Produtos Cerveja e Água do mesmo usuário</x:v>
+        <x:v>Conta aberta do usuário</x:v>
       </x:c>
       <x:c r="F79" s="29" t="str">
-        <x:v>Editar Água informando Nome="Cerveja"</x:v>
+        <x:v>Adicionar pedido usando ProdutoId inexistente</x:v>
       </x:c>
       <x:c r="G79" s="29" t="str">
-        <x:v>Result.IsFailed. A alteração não é persistida</x:v>
+        <x:v>Result.IsFailed. Nenhum pedido é persistido</x:v>
       </x:c>
       <x:c r="H79" s="29" t="str">
-        <x:v>RN-06</x:v>
+        <x:v>RN-16</x:v>
       </x:c>
       <x:c r="I79" s="29" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
       <x:c r="A80" s="15" t="str">
-        <x:v>CT79</x:v>
+        <x:v>CT85</x:v>
       </x:c>
       <x:c r="B80" s="15" t="str">
-        <x:v>Mesa</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C80" s="15" t="str">
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D80" s="15" t="str">
-        <x:v>Editar mesa de outro usuário</x:v>
+        <x:v>Remover pedido inexistente</x:v>
       </x:c>
       <x:c r="E80" s="15" t="str">
-        <x:v>Mesa pertence ao usuário B</x:v>
+        <x:v>Conta aberta sem o PedidoId informado</x:v>
       </x:c>
       <x:c r="F80" s="15" t="str">
-        <x:v>Usuário A tenta editar a mesa de B</x:v>
+        <x:v>Remover pedido usando identificador inexistente</x:v>
       </x:c>
       <x:c r="G80" s="15" t="str">
-        <x:v>Result.IsFailed. Registro não é alterado</x:v>
+        <x:v>Result.IsFailed. Pedidos existentes permanecem inalterados</x:v>
       </x:c>
       <x:c r="H80" s="15" t="str">
-        <x:v>RN-02</x:v>
+        <x:v>RN-14</x:v>
       </x:c>
       <x:c r="I80" s="15" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
       <x:c r="A81" s="22" t="str">
-        <x:v>CT80</x:v>
+        <x:v>CT86</x:v>
       </x:c>
       <x:c r="B81" s="22" t="str">
         <x:v>Garçom</x:v>
@@ -2982,27 +2982,27 @@
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D81" s="22" t="str">
-        <x:v>Excluir garçom de outro usuário</x:v>
+        <x:v>Listar garçons filtra por usuário</x:v>
       </x:c>
       <x:c r="E81" s="22" t="str">
-        <x:v>Garçom pertence ao usuário B</x:v>
+        <x:v>Um garçom do usuário A e outro do usuário B</x:v>
       </x:c>
       <x:c r="F81" s="22" t="str">
-        <x:v>Usuário A tenta excluir o garçom de B</x:v>
+        <x:v>Selecionar todos como usuário A</x:v>
       </x:c>
       <x:c r="G81" s="22" t="str">
-        <x:v>Result.IsFailed. Registro permanece persistido</x:v>
+        <x:v>Retorna somente o garçom do usuário A</x:v>
       </x:c>
       <x:c r="H81" s="22" t="str">
-        <x:v>RN-02</x:v>
+        <x:v>RN-01, RN-02</x:v>
       </x:c>
       <x:c r="I81" s="22" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
       <x:c r="A82" s="29" t="str">
-        <x:v>CT81</x:v>
+        <x:v>CT87</x:v>
       </x:c>
       <x:c r="B82" s="29" t="str">
         <x:v>Produto</x:v>
@@ -3011,637 +3011,529 @@
         <x:v>Aplicação</x:v>
       </x:c>
       <x:c r="D82" s="29" t="str">
-        <x:v>Excluir produto de outro usuário</x:v>
+        <x:v>Listar produtos filtra por usuário</x:v>
       </x:c>
       <x:c r="E82" s="29" t="str">
-        <x:v>Produto pertence ao usuário B</x:v>
+        <x:v>Um produto do usuário A e outro do usuário B</x:v>
       </x:c>
       <x:c r="F82" s="29" t="str">
-        <x:v>Usuário A tenta excluir o produto de B</x:v>
+        <x:v>Selecionar todos como usuário A</x:v>
       </x:c>
       <x:c r="G82" s="29" t="str">
-        <x:v>Result.IsFailed. Registro permanece persistido</x:v>
+        <x:v>Retorna somente o produto do usuário A</x:v>
       </x:c>
       <x:c r="H82" s="29" t="str">
-        <x:v>RN-02</x:v>
+        <x:v>RN-01, RN-02</x:v>
       </x:c>
       <x:c r="I82" s="29" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
       <x:c r="A83" s="45" t="str">
-        <x:v>CT82</x:v>
+        <x:v>CT88</x:v>
       </x:c>
       <x:c r="B83" s="45" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Mesa</x:v>
       </x:c>
       <x:c r="C83" s="45" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Integração</x:v>
       </x:c>
       <x:c r="D83" s="45" t="str">
-        <x:v>Fechar conta de outro usuário</x:v>
+        <x:v>Repositório de Mesa executa CRUD</x:v>
       </x:c>
       <x:c r="E83" s="45" t="str">
-        <x:v>Conta pertence ao usuário B</x:v>
+        <x:v>Banco de teste isolado</x:v>
       </x:c>
       <x:c r="F83" s="45" t="str">
-        <x:v>Usuário A tenta fechar a conta de B</x:v>
+        <x:v>Inserir, selecionar, editar e excluir uma mesa usando o repositório</x:v>
       </x:c>
       <x:c r="G83" s="45" t="str">
-        <x:v>Result.IsFailed. Conta permanece aberta</x:v>
+        <x:v>Todas as operações são persistidas e recuperadas corretamente</x:v>
       </x:c>
       <x:c r="H83" s="45" t="str">
-        <x:v>RN-02</x:v>
+        <x:v>RN-03, RN-04</x:v>
       </x:c>
       <x:c r="I83" s="45" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
       <x:c r="A84" s="49" t="str">
-        <x:v>CT83</x:v>
+        <x:v>CT89</x:v>
       </x:c>
       <x:c r="B84" s="49" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Garçom</x:v>
       </x:c>
       <x:c r="C84" s="49" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Integração</x:v>
       </x:c>
       <x:c r="D84" s="49" t="str">
-        <x:v>Adicionar pedido em conta inexistente</x:v>
+        <x:v>Repositório de Garçom executa CRUD</x:v>
       </x:c>
       <x:c r="E84" s="49" t="str">
-        <x:v>Produto válido do usuário</x:v>
+        <x:v>Banco de teste isolado</x:v>
       </x:c>
       <x:c r="F84" s="49" t="str">
-        <x:v>Adicionar pedido usando ContaId inexistente</x:v>
+        <x:v>Inserir, selecionar, editar e excluir um garçom usando o repositório</x:v>
       </x:c>
       <x:c r="G84" s="49" t="str">
-        <x:v>Result.IsFailed. Nenhum pedido é persistido</x:v>
+        <x:v>Todas as operações são persistidas e recuperadas corretamente</x:v>
       </x:c>
       <x:c r="H84" s="49" t="str">
-        <x:v>RN-02</x:v>
+        <x:v>RN-05</x:v>
       </x:c>
       <x:c r="I84" s="49" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
       <x:c r="A85" s="49" t="str">
-        <x:v>CT84</x:v>
+        <x:v>CT90</x:v>
       </x:c>
       <x:c r="B85" s="49" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Produto</x:v>
       </x:c>
       <x:c r="C85" s="49" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Integração</x:v>
       </x:c>
       <x:c r="D85" s="49" t="str">
-        <x:v>Adicionar pedido com produto inexistente</x:v>
+        <x:v>Repositório de Produto executa CRUD</x:v>
       </x:c>
       <x:c r="E85" s="49" t="str">
-        <x:v>Conta aberta do usuário</x:v>
+        <x:v>Banco de teste isolado</x:v>
       </x:c>
       <x:c r="F85" s="49" t="str">
-        <x:v>Adicionar pedido usando ProdutoId inexistente</x:v>
+        <x:v>Inserir, selecionar, editar e excluir um produto usando o repositório</x:v>
       </x:c>
       <x:c r="G85" s="49" t="str">
-        <x:v>Result.IsFailed. Nenhum pedido é persistido</x:v>
+        <x:v>Todas as operações são persistidas e recuperadas corretamente</x:v>
       </x:c>
       <x:c r="H85" s="49" t="str">
-        <x:v>RN-16</x:v>
+        <x:v>RN-06, RN-07</x:v>
       </x:c>
       <x:c r="I85" s="49" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
       <x:c r="A86" s="49" t="str">
-        <x:v>CT85</x:v>
+        <x:v>CT91</x:v>
       </x:c>
       <x:c r="B86" s="49" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Conta</x:v>
       </x:c>
       <x:c r="C86" s="49" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Integração</x:v>
       </x:c>
       <x:c r="D86" s="49" t="str">
-        <x:v>Remover pedido inexistente</x:v>
+        <x:v>Repositório de Conta persiste relacionamentos</x:v>
       </x:c>
       <x:c r="E86" s="49" t="str">
-        <x:v>Conta aberta sem o PedidoId informado</x:v>
+        <x:v>Banco isolado com mesa e garçom persistidos</x:v>
       </x:c>
       <x:c r="F86" s="49" t="str">
-        <x:v>Remover pedido usando identificador inexistente</x:v>
+        <x:v>Persistir conta e recarregar incluindo Mesa, Garçom e Pedidos</x:v>
       </x:c>
       <x:c r="G86" s="49" t="str">
-        <x:v>Result.IsFailed. Pedidos existentes permanecem inalterados</x:v>
+        <x:v>Conta e relacionamentos são recuperados corretamente</x:v>
       </x:c>
       <x:c r="H86" s="49" t="str">
-        <x:v>RN-14</x:v>
+        <x:v>RN-12</x:v>
       </x:c>
       <x:c r="I86" s="49" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
       <x:c r="A87" s="22" t="str">
-        <x:v>CT86</x:v>
+        <x:v>CT92</x:v>
       </x:c>
       <x:c r="B87" s="22" t="str">
-        <x:v>Garçom</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C87" s="22" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Integração</x:v>
       </x:c>
       <x:c r="D87" s="22" t="str">
-        <x:v>Listar garçons filtra por usuário</x:v>
+        <x:v>Repositório de Pedido persiste e remove pedido</x:v>
       </x:c>
       <x:c r="E87" s="22" t="str">
-        <x:v>Um garçom do usuário A e outro do usuário B</x:v>
+        <x:v>Banco isolado com conta aberta e produto</x:v>
       </x:c>
       <x:c r="F87" s="22" t="str">
-        <x:v>Selecionar todos como usuário A</x:v>
+        <x:v>Persistir pedido, recarregar e remover</x:v>
       </x:c>
       <x:c r="G87" s="22" t="str">
-        <x:v>Retorna somente o garçom do usuário A</x:v>
+        <x:v>Inclusão e remoção são refletidas no banco</x:v>
       </x:c>
       <x:c r="H87" s="22" t="str">
-        <x:v>RN-01, RN-02</x:v>
+        <x:v>RN-14, RN-15</x:v>
       </x:c>
       <x:c r="I87" s="22" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
       <x:c r="A88" s="29" t="str">
-        <x:v>CT87</x:v>
+        <x:v>CT93</x:v>
       </x:c>
       <x:c r="B88" s="29" t="str">
-        <x:v>Produto</x:v>
+        <x:v>Multi-tenancy</x:v>
       </x:c>
       <x:c r="C88" s="29" t="str">
-        <x:v>Aplicação</x:v>
+        <x:v>Integração</x:v>
       </x:c>
       <x:c r="D88" s="29" t="str">
-        <x:v>Listar produtos filtra por usuário</x:v>
+        <x:v>Filtros globais isolam todas as entidades por usuário</x:v>
       </x:c>
       <x:c r="E88" s="29" t="str">
-        <x:v>Um produto do usuário A e outro do usuário B</x:v>
+        <x:v>Banco isolado com registros equivalentes dos usuários A e B</x:v>
       </x:c>
       <x:c r="F88" s="29" t="str">
-        <x:v>Selecionar todos como usuário A</x:v>
+        <x:v>Consultar Mesas, Garçons, Produtos, Contas e Pedidos como usuário A</x:v>
       </x:c>
       <x:c r="G88" s="29" t="str">
-        <x:v>Retorna somente o produto do usuário A</x:v>
+        <x:v>Nenhuma consulta retorna registros do usuário B</x:v>
       </x:c>
       <x:c r="H88" s="29" t="str">
         <x:v>RN-01, RN-02</x:v>
       </x:c>
       <x:c r="I88" s="29" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
       <x:c r="A89" s="15" t="str">
-        <x:v>CT88</x:v>
+        <x:v>CT94</x:v>
       </x:c>
       <x:c r="B89" s="15" t="str">
-        <x:v>Mesa</x:v>
+        <x:v>Persistência</x:v>
       </x:c>
       <x:c r="C89" s="15" t="str">
         <x:v>Integração</x:v>
       </x:c>
       <x:c r="D89" s="15" t="str">
-        <x:v>Repositório de Mesa executa CRUD</x:v>
+        <x:v>Banco bloqueia exclusão de registros vinculados</x:v>
       </x:c>
       <x:c r="E89" s="15" t="str">
-        <x:v>Banco de teste isolado</x:v>
+        <x:v>Mesa, garçom e produto possuem vínculos persistidos</x:v>
       </x:c>
       <x:c r="F89" s="15" t="str">
-        <x:v>Inserir, selecionar, editar e excluir uma mesa usando o repositório</x:v>
+        <x:v>Tentar excluir cada registro diretamente pelo repositório</x:v>
       </x:c>
       <x:c r="G89" s="15" t="str">
-        <x:v>Todas as operações são persistidas e recuperadas corretamente</x:v>
+        <x:v>A integridade referencial impede exclusões que quebrariam o histórico</x:v>
       </x:c>
       <x:c r="H89" s="15" t="str">
-        <x:v>RN-03, RN-04</x:v>
+        <x:v>RN-08</x:v>
       </x:c>
       <x:c r="I89" s="15" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
       <x:c r="A90" s="22" t="str">
-        <x:v>CT89</x:v>
+        <x:v>CT95</x:v>
       </x:c>
       <x:c r="B90" s="22" t="str">
-        <x:v>Garçom</x:v>
+        <x:v>Pedido</x:v>
       </x:c>
       <x:c r="C90" s="22" t="str">
         <x:v>Integração</x:v>
       </x:c>
       <x:c r="D90" s="22" t="str">
-        <x:v>Repositório de Garçom executa CRUD</x:v>
+        <x:v>Snapshot é preservado após recarregar do banco</x:v>
       </x:c>
       <x:c r="E90" s="22" t="str">
-        <x:v>Banco de teste isolado</x:v>
+        <x:v>Pedido persistido com nome e preço do produto</x:v>
       </x:c>
       <x:c r="F90" s="22" t="str">
-        <x:v>Inserir, selecionar, editar e excluir um garçom usando o repositório</x:v>
+        <x:v>Editar o produto e recarregar o pedido em novo contexto</x:v>
       </x:c>
       <x:c r="G90" s="22" t="str">
-        <x:v>Todas as operações são persistidas e recuperadas corretamente</x:v>
+        <x:v>ProdutoNome e ProdutoPreco permanecem com os valores originais</x:v>
       </x:c>
       <x:c r="H90" s="22" t="str">
-        <x:v>RN-05</x:v>
+        <x:v>RN-17</x:v>
       </x:c>
       <x:c r="I90" s="22" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15" hidden="0" customHeight="1">
       <x:c r="A91" s="29" t="str">
-        <x:v>CT90</x:v>
+        <x:v>CT96</x:v>
       </x:c>
       <x:c r="B91" s="29" t="str">
-        <x:v>Produto</x:v>
+        <x:v>Faturamento</x:v>
       </x:c>
       <x:c r="C91" s="29" t="str">
         <x:v>Integração</x:v>
       </x:c>
       <x:c r="D91" s="29" t="str">
-        <x:v>Repositório de Produto executa CRUD</x:v>
+        <x:v>Consulta de faturamento usa data de fechamento e usuário</x:v>
       </x:c>
       <x:c r="E91" s="29" t="str">
-        <x:v>Banco de teste isolado</x:v>
+        <x:v>Contas abertas e fechadas em datas e usuários diferentes</x:v>
       </x:c>
       <x:c r="F91" s="29" t="str">
-        <x:v>Inserir, selecionar, editar e excluir um produto usando o repositório</x:v>
+        <x:v>Executar consulta diária para o usuário A</x:v>
       </x:c>
       <x:c r="G91" s="29" t="str">
-        <x:v>Todas as operações são persistidas e recuperadas corretamente</x:v>
+        <x:v>Retorna somente contas fechadas na data e pertencentes ao usuário A</x:v>
       </x:c>
       <x:c r="H91" s="29" t="str">
-        <x:v>RN-06, RN-07</x:v>
+        <x:v>RN-01, RN-02, RN-20</x:v>
       </x:c>
       <x:c r="I91" s="29" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="15" hidden="0" customHeight="1">
       <x:c r="A92" s="45" t="str">
-        <x:v>CT91</x:v>
+        <x:v>CT97</x:v>
       </x:c>
       <x:c r="B92" s="45" t="str">
-        <x:v>Conta</x:v>
+        <x:v>Mesa</x:v>
       </x:c>
       <x:c r="C92" s="45" t="str">
-        <x:v>Integração</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D92" s="45" t="str">
-        <x:v>Repositório de Conta persiste relacionamentos</x:v>
+        <x:v>CRUD completo de mesa</x:v>
       </x:c>
       <x:c r="E92" s="45" t="str">
-        <x:v>Banco isolado com mesa e garçom persistidos</x:v>
+        <x:v>Usuário autenticado</x:v>
       </x:c>
       <x:c r="F92" s="45" t="str">
-        <x:v>Persistir conta e recarregar incluindo Mesa, Garçom e Pedidos</x:v>
+        <x:v>Cadastrar, visualizar, editar e excluir uma mesa sem vínculos</x:v>
       </x:c>
       <x:c r="G92" s="45" t="str">
-        <x:v>Conta e relacionamentos são recuperados corretamente</x:v>
+        <x:v>Operações concluídas e refletidas na interface</x:v>
       </x:c>
       <x:c r="H92" s="45" t="str">
-        <x:v>RN-12</x:v>
+        <x:v>RN-03, RN-04</x:v>
       </x:c>
       <x:c r="I92" s="45" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15" hidden="0" customHeight="1">
       <x:c r="A93" s="49" t="str">
-        <x:v>CT92</x:v>
+        <x:v>CT98</x:v>
       </x:c>
       <x:c r="B93" s="49" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Garçom</x:v>
       </x:c>
       <x:c r="C93" s="49" t="str">
-        <x:v>Integração</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D93" s="49" t="str">
-        <x:v>Repositório de Pedido persiste e remove pedido</x:v>
+        <x:v>CRUD completo de garçom</x:v>
       </x:c>
       <x:c r="E93" s="49" t="str">
-        <x:v>Banco isolado com conta aberta e produto</x:v>
+        <x:v>Usuário autenticado</x:v>
       </x:c>
       <x:c r="F93" s="49" t="str">
-        <x:v>Persistir pedido, recarregar e remover</x:v>
+        <x:v>Cadastrar, visualizar, editar e excluir um garçom sem vínculos</x:v>
       </x:c>
       <x:c r="G93" s="49" t="str">
-        <x:v>Inclusão e remoção são refletidas no banco</x:v>
+        <x:v>Operações concluídas e refletidas na interface</x:v>
       </x:c>
       <x:c r="H93" s="49" t="str">
-        <x:v>RN-14, RN-15</x:v>
+        <x:v>RN-05</x:v>
       </x:c>
       <x:c r="I93" s="49" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A94" s="22" t="str">
-        <x:v>CT93</x:v>
+        <x:v>CT99</x:v>
       </x:c>
       <x:c r="B94" s="22" t="str">
-        <x:v>Multi-tenancy</x:v>
+        <x:v>Produto</x:v>
       </x:c>
       <x:c r="C94" s="22" t="str">
-        <x:v>Integração</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D94" s="22" t="str">
-        <x:v>Filtros globais isolam todas as entidades por usuário</x:v>
+        <x:v>CRUD completo de produto</x:v>
       </x:c>
       <x:c r="E94" s="22" t="str">
-        <x:v>Banco isolado com registros equivalentes dos usuários A e B</x:v>
+        <x:v>Usuário autenticado</x:v>
       </x:c>
       <x:c r="F94" s="22" t="str">
-        <x:v>Consultar Mesas, Garçons, Produtos, Contas e Pedidos como usuário A</x:v>
+        <x:v>Cadastrar, buscar, editar e excluir um produto sem vínculos</x:v>
       </x:c>
       <x:c r="G94" s="22" t="str">
-        <x:v>Nenhuma consulta retorna registros do usuário B</x:v>
+        <x:v>Operações concluídas e refletidas na interface</x:v>
       </x:c>
       <x:c r="H94" s="22" t="str">
-        <x:v>RN-01, RN-02</x:v>
+        <x:v>RN-06, RN-07</x:v>
       </x:c>
       <x:c r="I94" s="22" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A95" s="53" t="str">
-        <x:v>CT94</x:v>
+        <x:v>CT100</x:v>
       </x:c>
       <x:c r="B95" s="53" t="str">
-        <x:v>Persistência</x:v>
+        <x:v>Autenticação</x:v>
       </x:c>
       <x:c r="C95" s="53" t="str">
-        <x:v>Integração</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D95" s="53" t="str">
-        <x:v>Banco bloqueia exclusão de registros vinculados</x:v>
+        <x:v>Registrar e-mail já utilizado</x:v>
       </x:c>
       <x:c r="E95" s="53" t="str">
-        <x:v>Mesa, garçom e produto possuem vínculos persistidos</x:v>
+        <x:v>Usuário já registrado</x:v>
       </x:c>
       <x:c r="F95" s="53" t="str">
-        <x:v>Tentar excluir cada registro diretamente pelo repositório</x:v>
+        <x:v>Tentar registrar novamente com o mesmo e-mail</x:v>
       </x:c>
       <x:c r="G95" s="53" t="str">
-        <x:v>A integridade referencial impede exclusões que quebrariam o histórico</x:v>
+        <x:v>Validação exibida e nenhum segundo usuário é criado</x:v>
       </x:c>
       <x:c r="H95" s="53" t="str">
-        <x:v>RN-08</x:v>
+        <x:v>Funcionalidade: Autenticação</x:v>
       </x:c>
       <x:c r="I95" s="53" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A96" s="49" t="str">
-        <x:v>CT95</x:v>
+        <x:v>CT101</x:v>
       </x:c>
       <x:c r="B96" s="49" t="str">
-        <x:v>Pedido</x:v>
+        <x:v>Autenticação</x:v>
       </x:c>
       <x:c r="C96" s="49" t="str">
-        <x:v>Integração</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D96" s="49" t="str">
-        <x:v>Snapshot é preservado após recarregar do banco</x:v>
+        <x:v>Registrar com confirmação de senha diferente</x:v>
       </x:c>
       <x:c r="E96" s="49" t="str">
-        <x:v>Pedido persistido com nome e preço do produto</x:v>
+        <x:v>Nenhuma</x:v>
       </x:c>
       <x:c r="F96" s="49" t="str">
-        <x:v>Editar o produto e recarregar o pedido em novo contexto</x:v>
+        <x:v>Informar senha e confirmação diferentes e enviar</x:v>
       </x:c>
       <x:c r="G96" s="49" t="str">
-        <x:v>ProdutoNome e ProdutoPreco permanecem com os valores originais</x:v>
+        <x:v>Validação exibida e usuário não é criado</x:v>
       </x:c>
       <x:c r="H96" s="49" t="str">
-        <x:v>RN-17</x:v>
+        <x:v>Funcionalidade: Autenticação</x:v>
       </x:c>
       <x:c r="I96" s="49" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A97" s="53" t="str">
-        <x:v>CT96</x:v>
+        <x:v>CT102</x:v>
       </x:c>
       <x:c r="B97" s="53" t="str">
-        <x:v>Faturamento</x:v>
+        <x:v>Multi-tenancy</x:v>
       </x:c>
       <x:c r="C97" s="53" t="str">
-        <x:v>Integração</x:v>
+        <x:v>E2E</x:v>
       </x:c>
       <x:c r="D97" s="53" t="str">
-        <x:v>Consulta de faturamento usa data de fechamento e usuário</x:v>
+        <x:v>Usuário não visualiza dados de outro estabelecimento</x:v>
       </x:c>
       <x:c r="E97" s="53" t="str">
-        <x:v>Contas abertas e fechadas em datas e usuários diferentes</x:v>
+        <x:v>Usuários A e B possuem cadastros próprios</x:v>
       </x:c>
       <x:c r="F97" s="53" t="str">
-        <x:v>Executar consulta diária para o usuário A</x:v>
+        <x:v>Entrar como A e navegar por Mesas, Garçons, Produtos e Contas</x:v>
       </x:c>
       <x:c r="G97" s="53" t="str">
-        <x:v>Retorna somente contas fechadas na data e pertencentes ao usuário A</x:v>
+        <x:v>Somente dados do usuário A são exibidos</x:v>
       </x:c>
       <x:c r="H97" s="53" t="str">
-        <x:v>RN-01, RN-02, RN-20</x:v>
+        <x:v>RN-01, RN-02</x:v>
       </x:c>
       <x:c r="I97" s="53" t="str">
-        <x:v>A Fazer</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="15" hidden="0" customHeight="1">
-      <x:c r="A98" s="15" t="str">
-        <x:v>CT97</x:v>
-      </x:c>
-      <x:c r="B98" s="15" t="str">
-        <x:v>Mesa</x:v>
-      </x:c>
-      <x:c r="C98" s="15" t="str">
-        <x:v>E2E</x:v>
-      </x:c>
-      <x:c r="D98" s="15" t="str">
-        <x:v>CRUD completo de mesa</x:v>
-      </x:c>
-      <x:c r="E98" s="15" t="str">
-        <x:v>Usuário autenticado</x:v>
-      </x:c>
-      <x:c r="F98" s="15" t="str">
-        <x:v>Cadastrar, visualizar, editar e excluir uma mesa sem vínculos</x:v>
-      </x:c>
-      <x:c r="G98" s="15" t="str">
-        <x:v>Operações concluídas e refletidas na interface</x:v>
-      </x:c>
-      <x:c r="H98" s="15" t="str">
-        <x:v>RN-03, RN-04</x:v>
-      </x:c>
-      <x:c r="I98" s="15" t="str">
-        <x:v>A Fazer</x:v>
-      </x:c>
+      <x:c r="A98"/>
+      <x:c r="B98"/>
+      <x:c r="C98"/>
+      <x:c r="D98"/>
+      <x:c r="E98"/>
+      <x:c r="F98"/>
+      <x:c r="G98"/>
+      <x:c r="H98"/>
+      <x:c r="I98"/>
     </x:row>
     <x:row r="99" ht="15" hidden="0" customHeight="1">
-      <x:c r="A99" s="22" t="str">
-        <x:v>CT98</x:v>
-      </x:c>
-      <x:c r="B99" s="22" t="str">
-        <x:v>Garçom</x:v>
-      </x:c>
-      <x:c r="C99" s="22" t="str">
-        <x:v>E2E</x:v>
-      </x:c>
-      <x:c r="D99" s="22" t="str">
-        <x:v>CRUD completo de garçom</x:v>
-      </x:c>
-      <x:c r="E99" s="22" t="str">
-        <x:v>Usuário autenticado</x:v>
-      </x:c>
-      <x:c r="F99" s="22" t="str">
-        <x:v>Cadastrar, visualizar, editar e excluir um garçom sem vínculos</x:v>
-      </x:c>
-      <x:c r="G99" s="22" t="str">
-        <x:v>Operações concluídas e refletidas na interface</x:v>
-      </x:c>
-      <x:c r="H99" s="22" t="str">
-        <x:v>RN-05</x:v>
-      </x:c>
-      <x:c r="I99" s="22" t="str">
-        <x:v>A Fazer</x:v>
-      </x:c>
+      <x:c r="A99"/>
+      <x:c r="B99"/>
+      <x:c r="C99"/>
+      <x:c r="D99"/>
+      <x:c r="E99"/>
+      <x:c r="F99"/>
+      <x:c r="G99"/>
+      <x:c r="H99"/>
+      <x:c r="I99"/>
     </x:row>
     <x:row r="100" ht="15" hidden="0" customHeight="1">
-      <x:c r="A100" s="29" t="str">
-        <x:v>CT99</x:v>
-      </x:c>
-      <x:c r="B100" s="29" t="str">
-        <x:v>Produto</x:v>
-      </x:c>
-      <x:c r="C100" s="29" t="str">
-        <x:v>E2E</x:v>
-      </x:c>
-      <x:c r="D100" s="29" t="str">
-        <x:v>CRUD completo de produto</x:v>
-      </x:c>
-      <x:c r="E100" s="29" t="str">
-        <x:v>Usuário autenticado</x:v>
-      </x:c>
-      <x:c r="F100" s="29" t="str">
-        <x:v>Cadastrar, buscar, editar e excluir um produto sem vínculos</x:v>
-      </x:c>
-      <x:c r="G100" s="29" t="str">
-        <x:v>Operações concluídas e refletidas na interface</x:v>
-      </x:c>
-      <x:c r="H100" s="29" t="str">
-        <x:v>RN-06, RN-07</x:v>
-      </x:c>
-      <x:c r="I100" s="29" t="str">
-        <x:v>A Fazer</x:v>
-      </x:c>
+      <x:c r="A100"/>
+      <x:c r="B100"/>
+      <x:c r="C100"/>
+      <x:c r="D100"/>
+      <x:c r="E100"/>
+      <x:c r="F100"/>
+      <x:c r="G100"/>
+      <x:c r="H100"/>
+      <x:c r="I100"/>
     </x:row>
     <x:row r="101" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A101" s="57" t="str">
-        <x:v>CT100</x:v>
-      </x:c>
-      <x:c r="B101" s="57" t="str">
-        <x:v>Autenticação</x:v>
-      </x:c>
-      <x:c r="C101" s="57" t="str">
-        <x:v>E2E</x:v>
-      </x:c>
-      <x:c r="D101" s="57" t="str">
-        <x:v>Registrar e-mail já utilizado</x:v>
-      </x:c>
-      <x:c r="E101" s="57" t="str">
-        <x:v>Usuário já registrado</x:v>
-      </x:c>
-      <x:c r="F101" s="57" t="str">
-        <x:v>Tentar registrar novamente com o mesmo e-mail</x:v>
-      </x:c>
-      <x:c r="G101" s="57" t="str">
-        <x:v>Validação exibida e nenhum segundo usuário é criado</x:v>
-      </x:c>
-      <x:c r="H101" s="57" t="str">
-        <x:v>Funcionalidade: Autenticação</x:v>
-      </x:c>
-      <x:c r="I101" s="57" t="str">
-        <x:v>A Fazer</x:v>
-      </x:c>
+      <x:c r="A101"/>
+      <x:c r="B101"/>
+      <x:c r="C101"/>
+      <x:c r="D101"/>
+      <x:c r="E101"/>
+      <x:c r="F101"/>
+      <x:c r="G101"/>
+      <x:c r="H101"/>
+      <x:c r="I101"/>
     </x:row>
     <x:row r="102" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A102" s="57" t="str">
-        <x:v>CT101</x:v>
-      </x:c>
-      <x:c r="B102" s="57" t="str">
-        <x:v>Autenticação</x:v>
-      </x:c>
-      <x:c r="C102" s="57" t="str">
-        <x:v>E2E</x:v>
-      </x:c>
-      <x:c r="D102" s="57" t="str">
-        <x:v>Registrar com confirmação de senha diferente</x:v>
-      </x:c>
-      <x:c r="E102" s="57" t="str">
-        <x:v>Nenhuma</x:v>
-      </x:c>
-      <x:c r="F102" s="57" t="str">
-        <x:v>Informar senha e confirmação diferentes e enviar</x:v>
-      </x:c>
-      <x:c r="G102" s="57" t="str">
-        <x:v>Validação exibida e usuário não é criado</x:v>
-      </x:c>
-      <x:c r="H102" s="57" t="str">
-        <x:v>Funcionalidade: Autenticação</x:v>
-      </x:c>
-      <x:c r="I102" s="57" t="str">
-        <x:v>A Fazer</x:v>
-      </x:c>
+      <x:c r="A102"/>
+      <x:c r="B102"/>
+      <x:c r="C102"/>
+      <x:c r="D102"/>
+      <x:c r="E102"/>
+      <x:c r="F102"/>
+      <x:c r="G102"/>
+      <x:c r="H102"/>
+      <x:c r="I102"/>
     </x:row>
     <x:row r="103" ht="15" hidden="0" customHeight="1">
-      <x:c r="A103" s="22" t="str">
-        <x:v>CT102</x:v>
-      </x:c>
-      <x:c r="B103" s="22" t="str">
-        <x:v>Multi-tenancy</x:v>
-      </x:c>
-      <x:c r="C103" s="22" t="str">
-        <x:v>E2E</x:v>
-      </x:c>
-      <x:c r="D103" s="22" t="str">
-        <x:v>Usuário não visualiza dados de outro estabelecimento</x:v>
-      </x:c>
-      <x:c r="E103" s="22" t="str">
-        <x:v>Usuários A e B possuem cadastros próprios</x:v>
-      </x:c>
-      <x:c r="F103" s="22" t="str">
-        <x:v>Entrar como A e navegar por Mesas, Garçons, Produtos e Contas</x:v>
-      </x:c>
-      <x:c r="G103" s="22" t="str">
-        <x:v>Somente dados do usuário A são exibidos</x:v>
-      </x:c>
-      <x:c r="H103" s="22" t="str">
-        <x:v>RN-01, RN-02</x:v>
-      </x:c>
-      <x:c r="I103" s="22" t="str">
-        <x:v>A Fazer</x:v>
-      </x:c>
+      <x:c r="A103"/>
+      <x:c r="B103"/>
+      <x:c r="C103"/>
+      <x:c r="D103"/>
+      <x:c r="E103"/>
+      <x:c r="F103"/>
+      <x:c r="G103"/>
+      <x:c r="H103"/>
+      <x:c r="I103"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7332b69762b44234"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb13d52639764ec1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>